<commit_message>
se suben cv y skill de appdev
</commit_message>
<xml_diff>
--- a/SAT-SDMA-7 Perfiles.xlsx
+++ b/SAT-SDMA-7 Perfiles.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raquell.martinez\Documents\AISolutions\analyzeCV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2658ECC1-7A17-4441-A666-75F96C7D67DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48270E28-314C-46A5-AFAA-978C0A2F2BF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{D74C329F-941D-40F9-B295-21746B646AD6}"/>
+    <workbookView xWindow="0" yWindow="840" windowWidth="19360" windowHeight="10480" firstSheet="2" activeTab="2" xr2:uid="{D74C329F-941D-40F9-B295-21746B646AD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Líneas de acción" sheetId="5" state="hidden" r:id="rId1"/>
@@ -1934,7 +1934,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2087,6 +2087,12 @@
     <xf numFmtId="0" fontId="1" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2099,10 +2105,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3276,10 +3279,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C1" s="62" t="s">
+      <c r="C1" s="64" t="s">
         <v>368</v>
       </c>
-      <c r="D1" s="62"/>
+      <c r="D1" s="64"/>
       <c r="L1" s="16" t="s">
         <v>132</v>
       </c>
@@ -3435,7 +3438,7 @@
       </c>
     </row>
     <row r="3" spans="1:41" ht="90" x14ac:dyDescent="0.35">
-      <c r="B3" s="66" t="s">
+      <c r="B3" s="62" t="s">
         <v>66</v>
       </c>
       <c r="C3" s="21" t="s">
@@ -3795,7 +3798,7 @@
       </c>
     </row>
     <row r="6" spans="1:41" ht="150" x14ac:dyDescent="0.35">
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="62" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="21" t="s">
@@ -3915,7 +3918,7 @@
       </c>
     </row>
     <row r="7" spans="1:41" ht="150" x14ac:dyDescent="0.35">
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="62" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="21" t="s">
@@ -4035,7 +4038,7 @@
       </c>
     </row>
     <row r="8" spans="1:41" ht="140" x14ac:dyDescent="0.35">
-      <c r="B8" s="66" t="s">
+      <c r="B8" s="62" t="s">
         <v>55</v>
       </c>
       <c r="C8" s="21" t="s">
@@ -4155,7 +4158,7 @@
       </c>
     </row>
     <row r="9" spans="1:41" ht="140" x14ac:dyDescent="0.35">
-      <c r="B9" s="66" t="s">
+      <c r="B9" s="62" t="s">
         <v>57</v>
       </c>
       <c r="C9" s="21" t="s">
@@ -4275,7 +4278,7 @@
       </c>
     </row>
     <row r="10" spans="1:41" ht="70" x14ac:dyDescent="0.35">
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="62" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="21" t="s">
@@ -4747,7 +4750,7 @@
       </c>
     </row>
     <row r="14" spans="1:41" ht="140" x14ac:dyDescent="0.35">
-      <c r="B14" s="66" t="s">
+      <c r="B14" s="62" t="s">
         <v>60</v>
       </c>
       <c r="C14" s="21" t="s">
@@ -4867,7 +4870,7 @@
       </c>
     </row>
     <row r="15" spans="1:41" ht="140" x14ac:dyDescent="0.35">
-      <c r="B15" s="67" t="s">
+      <c r="B15" s="68" t="s">
         <v>59</v>
       </c>
       <c r="C15" s="21" t="s">
@@ -4988,7 +4991,7 @@
     </row>
     <row r="16" spans="1:41" ht="89" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="57"/>
-      <c r="B16" s="66" t="s">
+      <c r="B16" s="62" t="s">
         <v>64</v>
       </c>
       <c r="C16" s="21" t="s">
@@ -5109,7 +5112,7 @@
     </row>
     <row r="17" spans="1:41" ht="70" x14ac:dyDescent="0.35">
       <c r="A17" s="58"/>
-      <c r="B17" s="67" t="s">
+      <c r="B17" s="63" t="s">
         <v>62</v>
       </c>
       <c r="C17" s="21" t="s">
@@ -5472,7 +5475,7 @@
     </row>
     <row r="20" spans="1:41" ht="100" x14ac:dyDescent="0.35">
       <c r="A20" s="22"/>
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="68" t="s">
         <v>65</v>
       </c>
       <c r="C20" s="21" t="s">
@@ -5593,7 +5596,7 @@
     </row>
     <row r="21" spans="1:41" ht="140" x14ac:dyDescent="0.35">
       <c r="A21" s="22"/>
-      <c r="B21" s="21" t="s">
+      <c r="B21" s="68" t="s">
         <v>42</v>
       </c>
       <c r="C21" s="21" t="s">
@@ -5834,7 +5837,7 @@
       </c>
     </row>
     <row r="23" spans="1:41" ht="70" x14ac:dyDescent="0.35">
-      <c r="B23" s="21" t="s">
+      <c r="B23" s="68" t="s">
         <v>33</v>
       </c>
       <c r="C23" s="21" t="s">
@@ -13275,13 +13278,13 @@
       <c r="D1" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="64" t="s">
+      <c r="F1" s="66" t="s">
         <v>242</v>
       </c>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
     </row>
     <row r="2" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B2" s="39" t="s">
@@ -13293,11 +13296,11 @@
       <c r="D2" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B3" s="39" t="s">
@@ -13309,11 +13312,11 @@
       <c r="D3" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
+      <c r="J3" s="66"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B4" s="39" t="s">
@@ -13325,11 +13328,11 @@
       <c r="D4" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="64"/>
-      <c r="G4" s="64"/>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
-      <c r="J4" s="64"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
+      <c r="H4" s="66"/>
+      <c r="I4" s="66"/>
+      <c r="J4" s="66"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B5" s="39" t="s">
@@ -13341,11 +13344,11 @@
       <c r="D5" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="64"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
+      <c r="H5" s="66"/>
+      <c r="I5" s="66"/>
+      <c r="J5" s="66"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B6" s="39" t="s">
@@ -13357,11 +13360,11 @@
       <c r="D6" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="64"/>
-      <c r="G6" s="64"/>
-      <c r="H6" s="64"/>
-      <c r="I6" s="64"/>
-      <c r="J6" s="64"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="66"/>
+      <c r="J6" s="66"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B7" s="39" t="s">
@@ -13373,11 +13376,11 @@
       <c r="D7" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="64"/>
-      <c r="G7" s="64"/>
-      <c r="H7" s="64"/>
-      <c r="I7" s="64"/>
-      <c r="J7" s="64"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="66"/>
+      <c r="H7" s="66"/>
+      <c r="I7" s="66"/>
+      <c r="J7" s="66"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B9" s="37" t="s">
@@ -13560,13 +13563,13 @@
       <c r="D27" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="F27" s="65" t="s">
+      <c r="F27" s="67" t="s">
         <v>253</v>
       </c>
-      <c r="G27" s="65"/>
-      <c r="H27" s="65"/>
-      <c r="I27" s="65"/>
-      <c r="J27" s="65"/>
+      <c r="G27" s="67"/>
+      <c r="H27" s="67"/>
+      <c r="I27" s="67"/>
+      <c r="J27" s="67"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B28" s="39" t="s">
@@ -13578,13 +13581,13 @@
       <c r="D28" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="F28" s="65" t="s">
+      <c r="F28" s="67" t="s">
         <v>254</v>
       </c>
-      <c r="G28" s="65"/>
-      <c r="H28" s="65"/>
-      <c r="I28" s="65"/>
-      <c r="J28" s="65"/>
+      <c r="G28" s="67"/>
+      <c r="H28" s="67"/>
+      <c r="I28" s="67"/>
+      <c r="J28" s="67"/>
     </row>
     <row r="29" spans="2:10" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="39" t="s">
@@ -13596,13 +13599,13 @@
       <c r="D29" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="F29" s="63" t="s">
+      <c r="F29" s="65" t="s">
         <v>255</v>
       </c>
-      <c r="G29" s="63"/>
-      <c r="H29" s="63"/>
-      <c r="I29" s="63"/>
-      <c r="J29" s="63"/>
+      <c r="G29" s="65"/>
+      <c r="H29" s="65"/>
+      <c r="I29" s="65"/>
+      <c r="J29" s="65"/>
     </row>
     <row r="30" spans="2:10" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="39" t="s">
@@ -13614,13 +13617,13 @@
       <c r="D30" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="F30" s="63" t="s">
+      <c r="F30" s="65" t="s">
         <v>256</v>
       </c>
-      <c r="G30" s="63"/>
-      <c r="H30" s="63"/>
-      <c r="I30" s="63"/>
-      <c r="J30" s="63"/>
+      <c r="G30" s="65"/>
+      <c r="H30" s="65"/>
+      <c r="I30" s="65"/>
+      <c r="J30" s="65"/>
     </row>
     <row r="31" spans="2:10" ht="20" x14ac:dyDescent="0.35">
       <c r="B31" s="39" t="s">
@@ -13632,13 +13635,13 @@
       <c r="D31" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="F31" s="63" t="s">
+      <c r="F31" s="65" t="s">
         <v>257</v>
       </c>
-      <c r="G31" s="63"/>
-      <c r="H31" s="63"/>
-      <c r="I31" s="63"/>
-      <c r="J31" s="63"/>
+      <c r="G31" s="65"/>
+      <c r="H31" s="65"/>
+      <c r="I31" s="65"/>
+      <c r="J31" s="65"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B32" s="45"/>
@@ -14306,6 +14309,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100FC102D493A39B2419B6834134514A928" ma:contentTypeVersion="15" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="d01e0109bf6dea2fbada290e24a0079e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="882a8f42-f1f9-4ba8-a024-a9506b2a3f1b" xmlns:ns3="f3dc767a-0b06-462e-8350-fa01f76d53d6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5475975345732b2580ec347e706b0322" ns2:_="" ns3:_="">
     <xsd:import namespace="882a8f42-f1f9-4ba8-a024-a9506b2a3f1b"/>
@@ -14542,15 +14554,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -14564,6 +14567,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2F9F198-AAB3-4743-83B7-70E545DDE86B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E69E7B37-066B-460B-9CC0-96F997D136F5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14578,14 +14589,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2F9F198-AAB3-4743-83B7-70E545DDE86B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>